<commit_message>
chore: update data 2026-03-26
</commit_message>
<xml_diff>
--- a/data/downloads/AZ/FY_6_Final_ABA_FeeSchedule.xlsx
+++ b/data/downloads/AZ/FY_6_Final_ABA_FeeSchedule.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ahcccs.sharepoint.com/sites/DHCMReimbursement/Shared Documents/202510 FS Updates/Webfiles/Final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\106589\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{D2750756-526C-4C1D-8D96-9954D885E24E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33DC663C-CCFE-4A04-951E-636B2268798F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0103C218-7663-4755-BE5D-42F00DEFDFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{CA1D15D9-49A2-4D10-B07B-7F12D69B5255}"/>
+    <workbookView xWindow="-57720" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{CA1D15D9-49A2-4D10-B07B-7F12D69B5255}"/>
   </bookViews>
   <sheets>
-    <sheet name="FFY26 ABA FEE SCHEDULE 9.17.25" sheetId="1" r:id="rId1"/>
+    <sheet name="FFY26 ABA Fee Schedule 26.03.16" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FFY26 ABA FEE SCHEDULE 9.17.25'!$A$6:$F$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FFY26 ABA Fee Schedule 26.03.16'!$A$6:$F$63</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="34">
   <si>
     <t>Arizona Health Care Cost Containment System</t>
   </si>
@@ -134,7 +134,13 @@
     <t>ADAPTIVE BEHAVIOR TREATMENT BY PROFESSIONAL WITH GROUP USING AN ESTABLISHED PLAN, EACH 15 MINUTES</t>
   </si>
   <si>
-    <t>Last Updated on 9/17/25</t>
+    <t>Last Updated on 3/16/2026</t>
+  </si>
+  <si>
+    <t>TJ</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
@@ -244,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -284,9 +290,6 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -316,6 +319,100 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7612591</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EFD7E184-5880-F66C-776A-BC6C806D6148}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1259417" y="12840758"/>
+          <a:ext cx="7422091" cy="864659"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Note:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>* </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>The TJ modifier was added to the 97154 code for a highly specific group ABA model delivered in a community school setting as follows: ratio of ABA techs to patients in a community school setting must have multiple providers working with multiple patients, i.e. 2 providers with 3 children</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -635,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B031B761-EBD8-4846-AC0C-1B3D9648BB71}">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.26953125" style="2" bestFit="1" customWidth="1"/>
@@ -648,44 +745,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
     </row>
     <row r="4" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
     </row>
     <row r="5" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:6" s="9" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -731,10 +828,10 @@
       <c r="B8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="15"/>
+      <c r="C8" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="10"/>
       <c r="E8" s="13">
         <v>30.06</v>
       </c>
@@ -749,10 +846,10 @@
       <c r="B9" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="15"/>
+      <c r="D9" s="10"/>
       <c r="E9" s="13">
         <v>35.78</v>
       </c>
@@ -767,10 +864,10 @@
       <c r="B10" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="15"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="13">
         <v>44.73</v>
       </c>
@@ -785,8 +882,8 @@
       <c r="B11" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15">
+      <c r="C11" s="10"/>
+      <c r="D11" s="10">
         <v>12</v>
       </c>
       <c r="E11" s="13">
@@ -803,10 +900,10 @@
       <c r="B12" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="15">
+      <c r="C12" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="10">
         <v>12</v>
       </c>
       <c r="E12" s="13">
@@ -823,10 +920,10 @@
       <c r="B13" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="10">
         <v>12</v>
       </c>
       <c r="E13" s="13">
@@ -843,10 +940,10 @@
       <c r="B14" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="10">
         <v>12</v>
       </c>
       <c r="E14" s="13">
@@ -863,8 +960,8 @@
       <c r="B15" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
       <c r="E15" s="13">
         <v>21.49</v>
       </c>
@@ -879,10 +976,10 @@
       <c r="B16" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="15"/>
+      <c r="D16" s="10"/>
       <c r="E16" s="13">
         <v>21.49</v>
       </c>
@@ -897,10 +994,10 @@
       <c r="B17" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="15"/>
+      <c r="C17" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="10"/>
       <c r="E17" s="13">
         <v>25.58</v>
       </c>
@@ -915,10 +1012,10 @@
       <c r="B18" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="15"/>
+      <c r="D18" s="10"/>
       <c r="E18" s="13">
         <v>28.43</v>
       </c>
@@ -933,10 +1030,10 @@
       <c r="B19" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="15"/>
+      <c r="D19" s="10"/>
       <c r="E19" s="13">
         <v>28.43</v>
       </c>
@@ -951,8 +1048,8 @@
       <c r="B20" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15">
+      <c r="C20" s="10"/>
+      <c r="D20" s="10">
         <v>12</v>
       </c>
       <c r="E20" s="13">
@@ -969,10 +1066,10 @@
       <c r="B21" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="10">
         <v>12</v>
       </c>
       <c r="E21" s="13">
@@ -989,10 +1086,10 @@
       <c r="B22" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="15">
+      <c r="C22" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="10">
         <v>12</v>
       </c>
       <c r="E22" s="13">
@@ -1009,10 +1106,10 @@
       <c r="B23" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="C23" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="10">
         <v>12</v>
       </c>
       <c r="E23" s="13">
@@ -1029,10 +1126,10 @@
       <c r="B24" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="10">
         <v>12</v>
       </c>
       <c r="E24" s="13">
@@ -1049,8 +1146,8 @@
       <c r="B25" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
       <c r="E25" s="13">
         <v>17.91</v>
       </c>
@@ -1065,10 +1162,10 @@
       <c r="B26" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D26" s="15"/>
+      <c r="D26" s="10"/>
       <c r="E26" s="13">
         <v>17.91</v>
       </c>
@@ -1083,10 +1180,10 @@
       <c r="B27" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="15"/>
+      <c r="C27" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="10"/>
       <c r="E27" s="13">
         <v>21.32</v>
       </c>
@@ -1101,10 +1198,10 @@
       <c r="B28" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D28" s="15"/>
+      <c r="D28" s="10"/>
       <c r="E28" s="13">
         <v>23.69</v>
       </c>
@@ -1119,10 +1216,10 @@
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C29" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D29" s="15"/>
+      <c r="D29" s="10"/>
       <c r="E29" s="13">
         <v>23.69</v>
       </c>
@@ -1137,8 +1234,8 @@
       <c r="B30" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15">
+      <c r="C30" s="10"/>
+      <c r="D30" s="10">
         <v>12</v>
       </c>
       <c r="E30" s="13">
@@ -1155,10 +1252,10 @@
       <c r="B31" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="10">
         <v>12</v>
       </c>
       <c r="E31" s="13">
@@ -1175,10 +1272,10 @@
       <c r="B32" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="15">
+      <c r="C32" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="10">
         <v>12</v>
       </c>
       <c r="E32" s="13">
@@ -1195,10 +1292,10 @@
       <c r="B33" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="10">
         <v>12</v>
       </c>
       <c r="E33" s="13">
@@ -1215,10 +1312,10 @@
       <c r="B34" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="15" t="s">
+      <c r="C34" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D34" s="15">
+      <c r="D34" s="10">
         <v>12</v>
       </c>
       <c r="E34" s="13">
@@ -1235,8 +1332,8 @@
       <c r="B35" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
       <c r="E35" s="13">
         <v>4.4800000000000004</v>
       </c>
@@ -1251,10 +1348,10 @@
       <c r="B36" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="15" t="s">
+      <c r="C36" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D36" s="15"/>
+      <c r="D36" s="10"/>
       <c r="E36" s="13">
         <v>4.4800000000000004</v>
       </c>
@@ -1269,10 +1366,10 @@
       <c r="B37" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D37" s="15"/>
+      <c r="C37" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" s="10"/>
       <c r="E37" s="13">
         <v>5.33</v>
       </c>
@@ -1287,10 +1384,10 @@
       <c r="B38" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C38" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D38" s="15"/>
+      <c r="D38" s="10"/>
       <c r="E38" s="13">
         <v>5.92</v>
       </c>
@@ -1305,10 +1402,10 @@
       <c r="B39" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C39" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="15"/>
+      <c r="D39" s="10"/>
       <c r="E39" s="13">
         <v>5.92</v>
       </c>
@@ -1323,15 +1420,15 @@
       <c r="B40" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C40" s="15"/>
-      <c r="D40" s="15">
-        <v>12</v>
-      </c>
-      <c r="E40" s="13">
-        <v>4.99</v>
+      <c r="C40" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D40" s="10"/>
+      <c r="E40" s="13" t="s">
+        <v>33</v>
       </c>
       <c r="F40" s="14">
-        <v>45566</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
@@ -1341,10 +1438,8 @@
       <c r="B41" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C41" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D41" s="15">
+      <c r="C41" s="10"/>
+      <c r="D41" s="10">
         <v>12</v>
       </c>
       <c r="E41" s="13">
@@ -1361,14 +1456,14 @@
       <c r="B42" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" s="15">
+      <c r="C42" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D42" s="10">
         <v>12</v>
       </c>
       <c r="E42" s="13">
-        <v>5.95</v>
+        <v>4.99</v>
       </c>
       <c r="F42" s="14">
         <v>45566</v>
@@ -1381,14 +1476,14 @@
       <c r="B43" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C43" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D43" s="15">
+      <c r="C43" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D43" s="10">
         <v>12</v>
       </c>
       <c r="E43" s="13">
-        <v>6.61</v>
+        <v>5.95</v>
       </c>
       <c r="F43" s="14">
         <v>45566</v>
@@ -1401,10 +1496,10 @@
       <c r="B44" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D44" s="15">
+      <c r="C44" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" s="10">
         <v>12</v>
       </c>
       <c r="E44" s="13">
@@ -1416,15 +1511,19 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
+        <v>21</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" s="10">
+        <v>12</v>
+      </c>
       <c r="E45" s="13">
-        <v>25.05</v>
+        <v>6.61</v>
       </c>
       <c r="F45" s="14">
         <v>45566</v>
@@ -1437,10 +1536,8 @@
       <c r="B46" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C46" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D46" s="15"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
       <c r="E46" s="13">
         <v>25.05</v>
       </c>
@@ -1455,12 +1552,12 @@
       <c r="B47" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C47" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D47" s="15"/>
+      <c r="C47" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D47" s="10"/>
       <c r="E47" s="13">
-        <v>29.82</v>
+        <v>25.05</v>
       </c>
       <c r="F47" s="14">
         <v>45566</v>
@@ -1473,12 +1570,12 @@
       <c r="B48" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C48" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D48" s="15"/>
+      <c r="C48" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" s="10"/>
       <c r="E48" s="13">
-        <v>37.28</v>
+        <v>29.82</v>
       </c>
       <c r="F48" s="14">
         <v>45566</v>
@@ -1491,12 +1588,12 @@
       <c r="B49" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C49" s="15"/>
-      <c r="D49" s="15">
-        <v>12</v>
-      </c>
+      <c r="C49" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49" s="10"/>
       <c r="E49" s="13">
-        <v>27.72</v>
+        <v>37.28</v>
       </c>
       <c r="F49" s="14">
         <v>45566</v>
@@ -1509,10 +1606,8 @@
       <c r="B50" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C50" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D50" s="15">
+      <c r="C50" s="10"/>
+      <c r="D50" s="10">
         <v>12</v>
       </c>
       <c r="E50" s="13">
@@ -1529,14 +1624,14 @@
       <c r="B51" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C51" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D51" s="15">
+      <c r="C51" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D51" s="10">
         <v>12</v>
       </c>
       <c r="E51" s="13">
-        <v>33</v>
+        <v>27.72</v>
       </c>
       <c r="F51" s="14">
         <v>45566</v>
@@ -1549,14 +1644,14 @@
       <c r="B52" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C52" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D52" s="15">
+      <c r="C52" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" s="10">
         <v>12</v>
       </c>
       <c r="E52" s="13">
-        <v>41.25</v>
+        <v>33</v>
       </c>
       <c r="F52" s="14">
         <v>45566</v>
@@ -1564,15 +1659,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="13" t="s">
-        <v>26</v>
+        <v>23</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53" s="10">
+        <v>12</v>
+      </c>
+      <c r="E53" s="13">
+        <v>41.25</v>
       </c>
       <c r="F53" s="14">
         <v>45566</v>
@@ -1580,10 +1679,10 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C54" s="11"/>
       <c r="D54" s="11"/>
@@ -1596,15 +1695,15 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C55" s="15"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="13">
-        <v>6.26</v>
+        <v>28</v>
+      </c>
+      <c r="C55" s="11"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="13" t="s">
+        <v>26</v>
       </c>
       <c r="F55" s="14">
         <v>45566</v>
@@ -1617,10 +1716,8 @@
       <c r="B56" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C56" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D56" s="15"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="10"/>
       <c r="E56" s="13">
         <v>6.26</v>
       </c>
@@ -1635,12 +1732,12 @@
       <c r="B57" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C57" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D57" s="15"/>
+      <c r="C57" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57" s="10"/>
       <c r="E57" s="13">
-        <v>7.46</v>
+        <v>6.26</v>
       </c>
       <c r="F57" s="14">
         <v>45566</v>
@@ -1653,12 +1750,12 @@
       <c r="B58" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C58" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D58" s="15"/>
+      <c r="C58" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" s="10"/>
       <c r="E58" s="13">
-        <v>9.32</v>
+        <v>7.46</v>
       </c>
       <c r="F58" s="14">
         <v>45566</v>
@@ -1671,12 +1768,12 @@
       <c r="B59" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15">
-        <v>12</v>
-      </c>
+      <c r="C59" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D59" s="10"/>
       <c r="E59" s="13">
-        <v>6.93</v>
+        <v>9.32</v>
       </c>
       <c r="F59" s="14">
         <v>45566</v>
@@ -1689,10 +1786,8 @@
       <c r="B60" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C60" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D60" s="15">
+      <c r="C60" s="10"/>
+      <c r="D60" s="10">
         <v>12</v>
       </c>
       <c r="E60" s="13">
@@ -1709,14 +1804,14 @@
       <c r="B61" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C61" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D61" s="15">
+      <c r="C61" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D61" s="10">
         <v>12</v>
       </c>
       <c r="E61" s="13">
-        <v>8.25</v>
+        <v>6.93</v>
       </c>
       <c r="F61" s="14">
         <v>45566</v>
@@ -1729,32 +1824,52 @@
       <c r="B62" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C62" s="15" t="s">
+      <c r="C62" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62" s="10">
+        <v>12</v>
+      </c>
+      <c r="E62" s="13">
+        <v>8.25</v>
+      </c>
+      <c r="F62" s="14">
+        <v>45566</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C63" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D62" s="15">
-        <v>12</v>
-      </c>
-      <c r="E62" s="13">
+      <c r="D63" s="10">
+        <v>12</v>
+      </c>
+      <c r="E63" s="13">
         <v>10.31</v>
       </c>
-      <c r="F62" s="14">
-        <v>45566</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="2"/>
-      <c r="B66" s="1" t="s">
+      <c r="F63" s="14">
+        <v>45566</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="2"/>
+      <c r="B67" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C66" s="1"/>
-      <c r="D66" s="1"/>
-      <c r="F66" s="4"/>
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+      <c r="F67" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:F62" xr:uid="{A5997F72-BD31-44F9-87C2-03DC271A8B7D}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:F56">
-      <sortCondition ref="A6:A56"/>
+  <autoFilter ref="A6:F63" xr:uid="{A5997F72-BD31-44F9-87C2-03DC271A8B7D}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:F57">
+      <sortCondition ref="A6:A57"/>
     </sortState>
   </autoFilter>
   <mergeCells count="4">
@@ -1768,10 +1883,20 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Hyperlink xmlns="58d80952-9fc7-4439-aceb-6240e13bee17">
@@ -1791,18 +1916,9 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008189B72993416341A2A61CFCB66EEE3D" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="786006a6dd9b4bef0415ad58814c1d91">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="58d80952-9fc7-4439-aceb-6240e13bee17" xmlns:ns3="db31ca1b-3946-45b8-a263-034233bdb2d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a0b52c3a34e761563337a2af5449257e" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008189B72993416341A2A61CFCB66EEE3D" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="42e31d88fd7154a590b61c090dddd326">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="58d80952-9fc7-4439-aceb-6240e13bee17" xmlns:ns3="db31ca1b-3946-45b8-a263-034233bdb2d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="475718ef16372f821e943e2fd30f6c32" ns2:_="" ns3:_="">
     <xsd:import namespace="58d80952-9fc7-4439-aceb-6240e13bee17"/>
     <xsd:import namespace="db31ca1b-3946-45b8-a263-034233bdb2d8"/>
     <xsd:element name="properties">
@@ -2088,23 +2204,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C1D008C-9122-4A3A-98B2-882088FF8967}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="db31ca1b-3946-45b8-a263-034233bdb2d8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="58d80952-9fc7-4439-aceb-6240e13bee17"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B0EAE7C-EEC5-4436-8001-D309271D0CBE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2112,8 +2211,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C1D008C-9122-4A3A-98B2-882088FF8967}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="db31ca1b-3946-45b8-a263-034233bdb2d8"/>
+    <ds:schemaRef ds:uri="58d80952-9fc7-4439-aceb-6240e13bee17"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2A4427F-661A-4775-8DF8-A047ED73B753}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA5CA8F7-9D60-4FDE-BE6D-35C0664D9D8D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>

</xml_diff>